<commit_message>
fix rosstat labour force file link
</commit_message>
<xml_diff>
--- a/rosstat/testdata/labour_force.xlsx
+++ b/rosstat/testdata/labour_force.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="450" windowWidth="14985" windowHeight="12435" activeTab="1"/>
+    <workbookView activeTab="1" xWindow="60" yWindow="450" windowWidth="14985" windowHeight="12435"/>
   </bookViews>
   <sheets>
     <sheet name="Содержание" sheetId="16" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="321">
   <si>
     <t>Российская Федерация</t>
   </si>
@@ -2976,6 +2976,20 @@
   </si>
   <si>
     <r>
+      <t>июнь - август 2026</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="9"/>
+        <rFont val="Arial Cyr"/>
+        <charset val="204"/>
+      </rPr>
+      <t>2)</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>Обновлено:</t>
     </r>
     <r>
@@ -2985,7 +2999,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve"> 16.09.2026 г.</t>
+      <t xml:space="preserve"> 14.10.2026 г.</t>
     </r>
   </si>
 </sst>
@@ -3706,7 +3720,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3972,6 +3986,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4492,7 +4509,7 @@
     </row>
     <row r="18" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="39" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -4512,7 +4529,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.42578125" style="18" customWidth="1"/>
@@ -4521,10 +4538,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="105" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="104"/>
+      <c r="B1" s="105"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="34" t="s">
@@ -4548,36 +4565,36 @@
     </row>
     <row r="4" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:7" s="18" customFormat="1" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="110"/>
-      <c r="B5" s="112" t="s">
+      <c r="A5" s="111"/>
+      <c r="B5" s="113" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="114" t="s">
+      <c r="C5" s="115" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="115"/>
-      <c r="E5" s="112" t="s">
+      <c r="D5" s="116"/>
+      <c r="E5" s="113" t="s">
         <v>290</v>
       </c>
-      <c r="F5" s="106" t="s">
+      <c r="F5" s="107" t="s">
         <v>112</v>
       </c>
-      <c r="G5" s="108" t="s">
+      <c r="G5" s="109" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="111"/>
-      <c r="B6" s="113"/>
+      <c r="A6" s="112"/>
+      <c r="B6" s="114"/>
       <c r="C6" s="42" t="s">
         <v>114</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>115</v>
       </c>
-      <c r="E6" s="113"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="109"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="108"/>
+      <c r="G6" s="110"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="43" t="s">
@@ -7311,64 +7328,87 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="77" t="s">
+    <row r="131" spans="1:7" ht="13.5" x14ac:dyDescent="0.2">
+      <c r="A131" s="47" t="s">
         <v>172</v>
       </c>
-      <c r="B131" s="67">
+      <c r="B131" s="44">
         <v>76389.482000000004</v>
       </c>
-      <c r="C131" s="67">
+      <c r="C131" s="44">
         <v>74660.472999999998</v>
       </c>
-      <c r="D131" s="67">
+      <c r="D131" s="44">
         <v>1729.009</v>
       </c>
-      <c r="E131" s="68">
+      <c r="E131" s="45">
         <v>62.9</v>
       </c>
-      <c r="F131" s="68">
+      <c r="F131" s="45">
         <v>61.5</v>
       </c>
-      <c r="G131" s="69">
+      <c r="G131" s="46">
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="65" t="s">
+    <row r="132" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="77" t="s">
+        <v>173</v>
+      </c>
+      <c r="B132" s="67">
+        <v>76668.705000000002</v>
+      </c>
+      <c r="C132" s="67">
+        <v>75019.895999999993</v>
+      </c>
+      <c r="D132" s="67">
+        <v>1648.809</v>
+      </c>
+      <c r="E132" s="68">
+        <v>63.1</v>
+      </c>
+      <c r="F132" s="68">
+        <v>61.8</v>
+      </c>
+      <c r="G132" s="69">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="65" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="105" t="s">
+    <row r="134" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="106" t="s">
         <v>269</v>
       </c>
-      <c r="B133" s="105"/>
-      <c r="C133" s="105"/>
-      <c r="D133" s="105"/>
-      <c r="E133" s="105"/>
-      <c r="F133" s="105"/>
-      <c r="G133" s="105"/>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A134" s="74"/>
-      <c r="B134" s="84"/>
-      <c r="C134" s="84"/>
-      <c r="D134" s="85"/>
-      <c r="E134" s="83"/>
-      <c r="F134" s="83"/>
+      <c r="B134" s="106"/>
+      <c r="C134" s="106"/>
+      <c r="D134" s="106"/>
+      <c r="E134" s="106"/>
+      <c r="F134" s="106"/>
+      <c r="G134" s="106"/>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A135" s="74"/>
       <c r="B135" s="84"/>
       <c r="C135" s="84"/>
-      <c r="D135" s="84"/>
-      <c r="E135" s="84"/>
-      <c r="F135" s="84"/>
-      <c r="G135" s="84"/>
+      <c r="D135" s="85"/>
+      <c r="E135" s="83"/>
+      <c r="F135" s="83"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B136" s="84"/>
+      <c r="C136" s="84"/>
+      <c r="D136" s="84"/>
+      <c r="E136" s="84"/>
+      <c r="F136" s="84"/>
+      <c r="G136" s="84"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A133:G133"/>
+    <mergeCell ref="A134:G134"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
     <mergeCell ref="A1:B1"/>

</xml_diff>